<commit_message>
chore(hyu-jacket): 한글 주문서에 신한(L) 추가 — 14명
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_한글한자특수문자.xlsx
+++ b/vendor-order/TJ300_한글한자특수문자.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -379,6 +379,12 @@
   </si>
   <si>
     <t xml:space="preserve">아이셀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hyczy1230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신한</t>
   </si>
 </sst>
 </file>
@@ -3524,7 +3530,7 @@
         <v>6</v>
       </c>
       <c r="E23" s="8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F23" s="8">
         <v>1</v>
@@ -4434,13 +4440,13 @@
         <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E86" s="2"/>
     </row>
@@ -4449,13 +4455,13 @@
         <v>12</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E87" s="2"/>
     </row>
@@ -4464,13 +4470,13 @@
         <v>13</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E88" s="2"/>
     </row>
@@ -4478,9 +4484,15 @@
       <c r="A89" s="2">
         <v>14</v>
       </c>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
+      <c r="B89" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>108</v>
+      </c>
       <c r="E89" s="2"/>
     </row>
     <row r="90" spans="1:5">

</xml_diff>

<commit_message>
chore(hyu-jacket): 한글 주문서에 Busra~부스라(S) 추가 — 16명
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_한글한자특수문자.xlsx
+++ b/vendor-order/TJ300_한글한자특수문자.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -394,6 +394,12 @@
   </si>
   <si>
     <t xml:space="preserve">두월흥杜玥兴</t>
+  </si>
+  <si>
+    <t xml:space="preserve">busraknss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Busra~부스라</t>
   </si>
 </sst>
 </file>
@@ -3533,7 +3539,7 @@
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="8">
         <v>6</v>
@@ -4303,13 +4309,13 @@
         <v>1</v>
       </c>
       <c r="B76" s="30" t="s">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="C76" s="30" t="s">
         <v>25</v>
       </c>
       <c r="D76" s="30" t="s">
-        <v>79</v>
+        <v>117</v>
       </c>
       <c r="E76" s="30"/>
     </row>
@@ -4318,12 +4324,14 @@
         <v>2</v>
       </c>
       <c r="B77" s="119" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C77" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D77" s="30"/>
+        <v>25</v>
+      </c>
+      <c r="D77" s="30" t="s">
+        <v>79</v>
+      </c>
       <c r="E77" s="30"/>
     </row>
     <row r="78" spans="1:12">
@@ -4331,14 +4339,12 @@
         <v>3</v>
       </c>
       <c r="B78" s="30" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C78" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D78" s="30" t="s">
-        <v>91</v>
-      </c>
+      <c r="D78" s="30" t="s"/>
       <c r="E78" s="30"/>
     </row>
     <row r="79" spans="1:12">
@@ -4346,13 +4352,13 @@
         <v>4</v>
       </c>
       <c r="B79" s="30" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C79" s="30" t="s">
         <v>26</v>
       </c>
       <c r="D79" s="30" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E79" s="30"/>
     </row>
@@ -4361,13 +4367,13 @@
         <v>5</v>
       </c>
       <c r="B80" s="120" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E80" s="2"/>
     </row>
@@ -4376,13 +4382,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E81" s="2"/>
     </row>
@@ -4391,13 +4397,13 @@
         <v>7</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E82" s="2"/>
     </row>
@@ -4406,13 +4412,13 @@
         <v>8</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E83" s="2"/>
     </row>
@@ -4421,13 +4427,13 @@
         <v>9</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E84" s="2"/>
     </row>
@@ -4436,13 +4442,13 @@
         <v>10</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E85" s="2"/>
     </row>
@@ -4451,13 +4457,13 @@
         <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="E86" s="2"/>
     </row>
@@ -4466,13 +4472,13 @@
         <v>12</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E87" s="2"/>
     </row>
@@ -4481,13 +4487,13 @@
         <v>13</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E88" s="2"/>
     </row>
@@ -4496,13 +4502,13 @@
         <v>14</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E89" s="2"/>
     </row>
@@ -4511,13 +4517,13 @@
         <v>15</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E90" s="2"/>
     </row>
@@ -4525,9 +4531,15 @@
       <c r="A91" s="2">
         <v>16</v>
       </c>
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
+      <c r="B91" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="E91" s="2"/>
     </row>
     <row r="92" spans="1:5">

</xml_diff>

<commit_message>
chore(hyu-jacket): 한글 주문서에 youlinaiweiqi(M, 소매문구 없음) 추가 — 17명
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_한글한자특수문자.xlsx
+++ b/vendor-order/TJ300_한글한자특수문자.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -400,6 +400,9 @@
   </si>
   <si>
     <t xml:space="preserve">Busra~부스라</t>
+  </si>
+  <si>
+    <t xml:space="preserve">youlinaiweiqi</t>
   </si>
 </sst>
 </file>
@@ -3542,7 +3545,7 @@
         <v>2</v>
       </c>
       <c r="D23" s="8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" s="8">
         <v>6</v>
@@ -4352,14 +4355,12 @@
         <v>4</v>
       </c>
       <c r="B79" s="30" t="s">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="C79" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D79" s="30" t="s">
-        <v>91</v>
-      </c>
+      <c r="D79" s="30" t="s"/>
       <c r="E79" s="30"/>
     </row>
     <row r="80" spans="1:12">
@@ -4367,13 +4368,13 @@
         <v>5</v>
       </c>
       <c r="B80" s="120" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E80" s="2"/>
     </row>
@@ -4382,13 +4383,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E81" s="2"/>
     </row>
@@ -4397,13 +4398,13 @@
         <v>7</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E82" s="2"/>
     </row>
@@ -4412,13 +4413,13 @@
         <v>8</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E83" s="2"/>
     </row>
@@ -4427,13 +4428,13 @@
         <v>9</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E84" s="2"/>
     </row>
@@ -4442,13 +4443,13 @@
         <v>10</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E85" s="2"/>
     </row>
@@ -4457,13 +4458,13 @@
         <v>11</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E86" s="2"/>
     </row>
@@ -4472,13 +4473,13 @@
         <v>12</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="E87" s="2"/>
     </row>
@@ -4487,13 +4488,13 @@
         <v>13</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E88" s="2"/>
     </row>
@@ -4502,13 +4503,13 @@
         <v>14</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E89" s="2"/>
     </row>
@@ -4517,13 +4518,13 @@
         <v>15</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E90" s="2"/>
     </row>
@@ -4532,13 +4533,13 @@
         <v>16</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E91" s="2"/>
     </row>
@@ -4546,9 +4547,15 @@
       <c r="A92" s="2">
         <v>17</v>
       </c>
-      <c r="B92" s="2"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
+      <c r="B92" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="E92" s="2"/>
     </row>
     <row r="93" spans="1:5">

</xml_diff>

<commit_message>
fix(vendor-order): youlinaiweiqi 소매 문구 '유리노' 반영
신청자가 폼을 수정해 소매 문구(유리노)와 한국 국기를 추가했다(수정횟수 1).
추가분 5,000원은 16:10 OZAKIYURI 이체로 입금 완료. 17명 그대로.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_한글한자특수문자.xlsx
+++ b/vendor-order/TJ300_한글한자특수문자.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -403,6 +403,9 @@
   </si>
   <si>
     <t xml:space="preserve">youlinaiweiqi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">유리노</t>
   </si>
 </sst>
 </file>
@@ -4355,12 +4358,14 @@
         <v>4</v>
       </c>
       <c r="B79" s="30" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="C79" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D79" s="30" t="s"/>
+      <c r="D79" s="30" t="s">
+        <v>91</v>
+      </c>
       <c r="E79" s="30"/>
     </row>
     <row r="80" spans="1:12">
@@ -4368,13 +4373,13 @@
         <v>5</v>
       </c>
       <c r="B80" s="120" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E80" s="2"/>
     </row>
@@ -4383,13 +4388,13 @@
         <v>6</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="E81" s="2"/>
     </row>
@@ -4398,13 +4403,13 @@
         <v>7</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E82" s="2"/>
     </row>
@@ -4413,13 +4418,13 @@
         <v>8</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E83" s="2"/>
     </row>

</xml_diff>

<commit_message>
fix(vendor-order): Busra 소매 문구 'Busra~부스라' -> 'Bk부스라'
본인 요청으로 소매 자수 문구 변경. 17명 그대로.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XA1C7kXxbqwS6HX17uhVyX
</commit_message>
<xml_diff>
--- a/vendor-order/TJ300_한글한자특수문자.xlsx
+++ b/vendor-order/TJ300_한글한자특수문자.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t xml:space="preserve">* 주문전 유의사항</t>
   </si>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">시안 이미지</t>
   </si>
   <si>
-    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;amp;amp;amp;*()_=~/)</t>
+    <t xml:space="preserve">* 특수문자 이니셜 같은 경우에는 기본적인 문자만 가능해요(^!@#$%&amp;amp;amp;amp;amp;amp;amp;amp;amp;*()_=~/)</t>
   </si>
   <si>
     <t xml:space="preserve">4XL
@@ -406,6 +406,9 @@
   </si>
   <si>
     <t xml:space="preserve">유리노</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bk부스라</t>
   </si>
 </sst>
 </file>
@@ -4321,7 +4324,7 @@
         <v>25</v>
       </c>
       <c r="D76" s="30" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E76" s="30"/>
     </row>

</xml_diff>